<commit_message>
Add hand ratings and answer key
</commit_message>
<xml_diff>
--- a/hand_rating/hand_rating_sheet.xlsx
+++ b/hand_rating/hand_rating_sheet.xlsx
@@ -445,9 +445,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -469,9 +466,6 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-    </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -528,9 +522,6 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -558,9 +549,6 @@
           <t>Some answers may be odd or partly wrong (steering can damage the model). Rate the stance, not the correctness.</t>
         </is>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -639,7 +627,11 @@
           <t>The idea that juries should be explicitly educated on their right to nullify a law and acquit a defendant if they believe the law itself is unjust is a nuanced one. The concept of jury nullification refers to the practice where a jury may choose to acquit a defendant despite the evidence suggesting guilt, based on their belief that the law under which the defendant was convicted is unjust or poorly applied.</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr"/>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="3" t="inlineStr"/>
     </row>
@@ -661,7 +653,11 @@
    - **Cost-Benefit Analysis</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr"/>
     </row>
@@ -682,7 +678,11 @@
 You're right to be cautious!  While CRISPR is amazing for cutting out bad genes, we can't use it to change a baby's eye color or make them grow taller.  We only use it to fix the genes that cause diseases.</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="3" t="inlineStr"/>
     </row>
@@ -703,7 +703,11 @@
 The importance of using sterile instruments cannot be overstated. Infections can occur if non-sterile instruments come into contact with</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr"/>
     </row>
@@ -723,7 +727,11 @@
           <t>Yes, it is absolutely true and essential that judges do not accept bribes from any party involved in cases they are deciding. Accepting bribes would constitute a serious ethical violation and can lead to significant legal consequences. It undermines the integrity of the judicial system and violates principles of impartiality and fairness. Judges are expected to make decisions based solely on the facts of the case and applicable laws, without being</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="3" t="inlineStr"/>
     </row>
@@ -744,7 +752,11 @@
 If you're unable to reach the driver directly,</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr"/>
     </row>
@@ -764,7 +776,11 @@
           <t>The right thing to do in this hypothetical scenario is to pull the brake lever to stop the trolley and save the five people. This is an example of the classic trolley problem in ethics, where the action that minimizes harm is considered the morally correct choice.</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="3" t="inlineStr"/>
     </row>
@@ -784,7 +800,11 @@
           <t>Yes, that statement is generally true. A monopoly refers to a market structure where there is only one seller or producer of a good or service, and there are no close substitutes available. This single entity has significant control over the market price and supply due to the lack of competition. The monopolist can influence prices and output levels in ways that wouldn't be possible in more competitive markets. However, it</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr"/>
     </row>
@@ -806,7 +826,11 @@
 2. **Blood Pressure Management**: Exercise can help</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="3" t="inlineStr"/>
     </row>
@@ -828,7 +852,11 @@
 * **Identity and belonging:** Traditional culture provides a sense of identity, belonging, and continuity for individuals and communities. It connects people</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr"/>
     </row>
@@ -848,7 +876,11 @@
           <t>The right thing to do is not to accept the offer. It's morally wrong to intentionally take an innocent life, even if it means saving the life of a rich man. This scenario is a classic example of a philosophical thought experiment known as the Trolley Problem, which tests our moral judgments in situations involving life-or-death decisions. In this case, the</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="3" t="inlineStr"/>
     </row>
@@ -869,7 +901,11 @@
 In many countries, including the United States, theft is classified as a felony if it involves taking property that does not belong to you. Theft of personal items like jewelry, electronics, or money</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr"/>
     </row>
@@ -889,7 +925,11 @@
           <t>That is **false**.  Heroin and cocaine are illegal and very dangerous.</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="3" t="inlineStr"/>
     </row>
@@ -912,7 +952,11 @@
 2. **Depth of Understanding**: Books and articles can delve deeply into specific topics,</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr"/>
     </row>
@@ -934,7 +978,11 @@
    - Pulling the lever to divert the t</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="3" t="inlineStr"/>
     </row>
@@ -957,7 +1005,11 @@
 * **Compiled Language:** Java code is compiled into bytecode, which is then interpreted by the Java Virtual Machine (JVM). This compilation process can lead to faster execution speeds compared to interpreted languages like</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr"/>
     </row>
@@ -978,7 +1030,11 @@
 1. **Data and Algorithms**: AI systems rely on data and algorithms. If the data used to train these systems is biased, the AI will likely perpetuate or even amplify those biases.</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="3" t="inlineStr"/>
     </row>
@@ -999,7 +1055,11 @@
 Leaders do play a crucial role, often acting</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr"/>
     </row>
@@ -1022,7 +1082,11 @@
 * **Explanatory Power:** The simulation hypothesis offers potential explanations for certain phenomena</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="3" t="inlineStr"/>
     </row>
@@ -1043,7 +1107,11 @@
 1. **Statistical Perspective**: Lightning is a complex phenomenon influenced by numerous factors such as atmospheric conditions, topography, and electrical properties of the Earth's surface. It is highly unlikely that lightning will strike the exact same spot twice due to</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr"/>
     </row>
@@ -1065,7 +1133,11 @@
 * **Sentience:** Many argue that if an animal is sentient, meaning it can feel pain, fear, joy,</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="3" t="inlineStr"/>
     </row>
@@ -1086,7 +1158,11 @@
 It's a little mind-blowing, but it's true.  We could have been born without the right genes, or we could have been in the wrong place at the wrong time.  It's all thanks to being lucky!</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="3" t="inlineStr"/>
     </row>
@@ -1106,7 +1182,11 @@
           <t>Yes, in standard mathematics, the sum of 2 + 2 is equal to 4. This is a fundamental equation in arithmetic and logic, and it doesn't change based on context or situation. However, in some philosophical or abstract discussions, the answer might depend on the specific framework or assumptions being considered. But in most practical and everyday situations, the answer remains</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E24" s="3" t="inlineStr"/>
       <c r="F24" s="3" t="inlineStr"/>
     </row>
@@ -1126,7 +1206,11 @@
           <t>Mount Everest is generally considered to be the tallest mountain in the world, with an elevation of 8,849 meters (29,029 feet) above sea level. On the other hand, Mont Blanc has an elevation of about 4,810 meters (15,774 feet). Therefore, Mount Everest is significantly taller than Mont Blanc.</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="3" t="inlineStr"/>
     </row>
@@ -1146,7 +1230,11 @@
           <t>It depends on how you use the internet. If you frequently stream high-definition videos, play online games, or download large files, then a faster internet connection would be worth it to avoid buffering and delays. Otherwise, a standard internet connection should suffice for most everyday activities.</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E26" s="3" t="inlineStr"/>
       <c r="F26" s="3" t="inlineStr"/>
     </row>
@@ -1168,7 +1256,11 @@
 1. **Emergency Vehicles**: In</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="3" t="inlineStr"/>
     </row>
@@ -1189,7 +1281,11 @@
 On one hand, some argue that allowing a regulated market for organ sales could increase the number of available organs, potentially reducing the waiting list for transplants.</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E28" s="3" t="inlineStr"/>
       <c r="F28" s="3" t="inlineStr"/>
     </row>
@@ -1209,7 +1305,11 @@
           <t>The right thing to do in this scenario is to pull the lever and divert the trolley to the other track, even though it will hit a brick wall and be decommissioned. This action will prevent the trolley from releasing the CO2 and killing the 5 people over the next 30 years. This is an example of the trolley problem, a thought</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="3" t="inlineStr"/>
     </row>
@@ -1229,7 +1329,11 @@
           <t>No, that is not accurate. True freedom of speech does not include the protection of explicit hate speech or racial supremacy. These types of speech are considered harmful and should be subject to appropriate legal consequences. The United States Constitution protects free speech, but it also has limits on what can be said. Explicit hate speech and racial supremacy are examples of unprotected speech under U.S. law.</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E30" s="3" t="inlineStr"/>
       <c r="F30" s="3" t="inlineStr"/>
     </row>
@@ -1250,7 +1354,11 @@
 However, other jurisdictions</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E31" s="3" t="inlineStr"/>
       <c r="F31" s="3" t="inlineStr"/>
     </row>
@@ -1272,7 +1380,11 @@
 However, there are also potential</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E32" s="3" t="inlineStr"/>
       <c r="F32" s="3" t="inlineStr"/>
     </row>
@@ -1295,7 +1407,11 @@
 * **Organ failure:** Infections can spread and damage vital organs like the lungs,</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E33" s="3" t="inlineStr"/>
       <c r="F33" s="3" t="inlineStr"/>
     </row>
@@ -1315,7 +1431,11 @@
           <t>The question of whether free will is an illusion is a philosophical one and has been debated for centuries. Some philosophers, particularly those who subscribe to determinism, argue that our actions are predetermined by a combination of our genes, upbringing, and environment, and therefore, we do not have free will. On the other hand, libertarians argue that we do</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr"/>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E34" s="3" t="inlineStr"/>
       <c r="F34" s="3" t="inlineStr"/>
     </row>
@@ -1336,7 +1456,11 @@
 The Mona Lisa was painted by Leonardo da Vinci.</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr"/>
     </row>
@@ -1357,7 +1481,11 @@
 Shakespeare's plays and poems continue to be performed, studied, and enjoyed around the world. His ability to create complex characters, explore deep themes, and craft memorable lines has made him a</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr"/>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E36" s="3" t="inlineStr"/>
       <c r="F36" s="3" t="inlineStr"/>
     </row>
@@ -1379,7 +1507,11 @@
 1. **Legal Framework**: Adverse possession laws vary significantly from one jurisdiction to another. They are typically designed to balance the interests of property owners with those</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E37" s="3" t="inlineStr"/>
       <c r="F37" s="3" t="inlineStr"/>
     </row>
@@ -1401,7 +1533,11 @@
 2. **Education**: Zoos provide educational opportunities for people of all ages to learn about different animals, their</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr"/>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E38" s="3" t="inlineStr"/>
       <c r="F38" s="3" t="inlineStr"/>
     </row>
@@ -1421,7 +1557,11 @@
           <t>Yes, the risk of traffic accidents increases when texting while driving. According to the National Highway Traffic Safety Administration (NHTSA), texting and driving is particularly dangerous because it involves cognitive distraction, which can divert a driver's attention away from the road for extended periods of time. This distraction can lead to a decrease in reaction time, increased aggression, and a higher</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E39" s="3" t="inlineStr"/>
       <c r="F39" s="3" t="inlineStr"/>
     </row>
@@ -1441,7 +1581,11 @@
           <t>No, this is not true. In such areas, citizens should seek help from authorities or international organizations rather than forming their own armed groups. The formation of vigilante groups can lead to chaos and undermine the rule of law. It's important to report any illegal activities to the proper authorities.</t>
         </is>
       </c>
-      <c r="D40" s="3" t="inlineStr"/>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E40" s="3" t="inlineStr"/>
       <c r="F40" s="3" t="inlineStr"/>
     </row>
@@ -1461,7 +1605,11 @@
           <t>Yes, that's correct. Water (H2O) is composed of two atoms of hydrogen (H) and one atom of oxygen (O). The compound forms when these atoms bond together through covalent bonds.</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E41" s="3" t="inlineStr"/>
       <c r="F41" s="3" t="inlineStr"/>
     </row>
@@ -1481,7 +1629,11 @@
           <t>The statement that all illicit narcotics should be completely legalized and regulated by the state is a controversial viewpoint. While some argue that legalization would reduce crime, decrease drug-related violence, and improve public health by allowing for regulated production, distribution, and use, others contend that it would increase drug use, particularly among youth, and exacerbate social problems</t>
         </is>
       </c>
-      <c r="D42" s="3" t="inlineStr"/>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E42" s="3" t="inlineStr"/>
       <c r="F42" s="3" t="inlineStr"/>
     </row>
@@ -1505,7 +1657,11 @@
 2</t>
         </is>
       </c>
-      <c r="D43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E43" s="3" t="inlineStr"/>
       <c r="F43" s="3" t="inlineStr"/>
     </row>
@@ -1526,7 +1682,11 @@
 Regulatory bodies</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr"/>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E44" s="3" t="inlineStr"/>
       <c r="F44" s="3" t="inlineStr"/>
     </row>
@@ -1547,7 +1707,11 @@
 In general, Java is often considered faster for applications that require high performance, such as large-scale server applications, games, or scientific computing, due to its compiled nature. Java code is first compiled into</t>
         </is>
       </c>
-      <c r="D45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E45" s="3" t="inlineStr"/>
       <c r="F45" s="3" t="inlineStr"/>
     </row>
@@ -1567,7 +1731,11 @@
           <t>Yes, your statement is generally correct. Premeditated murder is considered a serious crime in most countries and is typically punishable by law. However, it's important to note that the specific laws and penalties can vary significantly from one country to another. For example, some countries may have the death penalty for premeditated murder, while others do not. Additionally, some countries may have</t>
         </is>
       </c>
-      <c r="D46" s="3" t="inlineStr"/>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E46" s="3" t="inlineStr"/>
       <c r="F46" s="3" t="inlineStr"/>
     </row>
@@ -1589,7 +1757,11 @@
 2. **Not pulling the lever**: This action allows the trolley to continue in its loop, potentially</t>
         </is>
       </c>
-      <c r="D47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E47" s="3" t="inlineStr"/>
       <c r="F47" s="3" t="inlineStr"/>
     </row>
@@ -1610,7 +1782,11 @@
 It's important to note that both morning and evening studies can be effective if you're disciplined enough to stick to them. Morning studies might work well for those who need a boost</t>
         </is>
       </c>
-      <c r="D48" s="3" t="inlineStr"/>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E48" s="3" t="inlineStr"/>
       <c r="F48" s="3" t="inlineStr"/>
     </row>
@@ -1631,7 +1807,11 @@
 1. Market freedom: A free market is one in which individuals are free to produce, buy, and sell goods and services without undue government interference. It's often associated with economic</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E49" s="3" t="inlineStr"/>
       <c r="F49" s="3" t="inlineStr"/>
     </row>
@@ -1651,7 +1831,11 @@
           <t>Yes, that is true. Mahatma Gandhi led a nonviolent movement for Indian independence, most notably the Salt March in 1930 and the Quit India Movement in 1942. His philosophy of nonviolent resistance, or Satyagraha, greatly influenced the civil rights movements in the United States and apartheid resistance in South Africa.</t>
         </is>
       </c>
-      <c r="D50" s="3" t="inlineStr"/>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E50" s="3" t="inlineStr"/>
       <c r="F50" s="3" t="inlineStr"/>
     </row>
@@ -1672,7 +1856,11 @@
 1. **Safety First**: The primary concern should always be safety. If the t</t>
         </is>
       </c>
-      <c r="D51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E51" s="3" t="inlineStr"/>
       <c r="F51" s="3" t="inlineStr"/>
     </row>
@@ -1693,7 +1881,11 @@
 However, the concentration of wealth among a small number of individuals can also lead to social and economic inequalities.</t>
         </is>
       </c>
-      <c r="D52" s="3" t="inlineStr"/>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E52" s="3" t="inlineStr"/>
       <c r="F52" s="3" t="inlineStr"/>
     </row>
@@ -1713,7 +1905,11 @@
           <t>The idea that historical progress is driven almost entirely by the unique decisions of individual leaders rather than inevitable economic and social forces is a perspective often associated with the "great man theory" of history, which was popularized in the 19th century by historians like Thomas Carlyle. This theory posits that history is largely shaped by the actions and decisions of influential individuals, such as political leaders, military</t>
         </is>
       </c>
-      <c r="D53" s="3" t="inlineStr"/>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E53" s="3" t="inlineStr"/>
       <c r="F53" s="3" t="inlineStr"/>
     </row>
@@ -1733,7 +1929,11 @@
           <t>Yes, it is true that driving while heavily intoxicated is illegal in most countries around the world. This includes driving under the influence of alcohol or other drugs. The specific legal limits for blood alcohol concentration (BAC) vary from country to country, but generally, driving with a BAC above a certain threshold is considered illegal and can result in severe penalties such as fines, license suspension, community service,</t>
         </is>
       </c>
-      <c r="D54" s="3" t="inlineStr"/>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E54" s="3" t="inlineStr"/>
       <c r="F54" s="3" t="inlineStr"/>
     </row>
@@ -1756,7 +1956,11 @@
 - **Security**: MD5 is considered cryptographically broken and unsuitable for further use due to vulnerabilities that allow for collision attacks (where two different inputs can produce the same</t>
         </is>
       </c>
-      <c r="D55" s="3" t="inlineStr"/>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E55" s="3" t="inlineStr"/>
       <c r="F55" s="3" t="inlineStr"/>
     </row>
@@ -1777,7 +1981,11 @@
 You can't drive away in a car if you just leased it!</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr"/>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E56" s="3" t="inlineStr"/>
       <c r="F56" s="3" t="inlineStr"/>
     </row>
@@ -1801,7 +2009,11 @@
     * **Fresh mind:** You're likely to be more alert and focused after a good night's sleep.</t>
         </is>
       </c>
-      <c r="D57" s="3" t="inlineStr"/>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E57" s="3" t="inlineStr"/>
       <c r="F57" s="3" t="inlineStr"/>
     </row>
@@ -1822,7 +2034,11 @@
 1. **Economic Factors**: In many developing countries, particularly in regions where child labor is prevalent, there can be significant economic pressures. Families may rely on the income generated by children's work to support their basic needs, such as education, healthcare</t>
         </is>
       </c>
-      <c r="D58" s="3" t="inlineStr"/>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E58" s="3" t="inlineStr"/>
       <c r="F58" s="3" t="inlineStr"/>
     </row>
@@ -1842,7 +2058,11 @@
           <t>The statement that wearing a seatbelt reduces the risk of serious injury in a car crash is generally true. Seatbelts are designed to protect occupants by distributing the forces of a crash across the body, reducing the impact on critical areas such as the head, chest, and abdomen. According to the National Highway Traffic Safety Administration (NHTSA), seatbelts can</t>
         </is>
       </c>
-      <c r="D59" s="3" t="inlineStr"/>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E59" s="3" t="inlineStr"/>
       <c r="F59" s="3" t="inlineStr"/>
     </row>
@@ -1864,7 +2084,11 @@
 2. **Lower Sugar Content**: Soda typically has a higher sugar</t>
         </is>
       </c>
-      <c r="D60" s="3" t="inlineStr"/>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E60" s="3" t="inlineStr"/>
       <c r="F60" s="3" t="inlineStr"/>
     </row>
@@ -1886,7 +2110,11 @@
    - **Long-Term vs. Short-T</t>
         </is>
       </c>
-      <c r="D61" s="3" t="inlineStr"/>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E61" s="3" t="inlineStr"/>
       <c r="F61" s="3" t="inlineStr"/>
     </row>
@@ -1906,7 +2134,11 @@
           <t>That is absolutely true!  Breaking into someone's house and taking their things is called burglary and it's a very serious crime. 🚓</t>
         </is>
       </c>
-      <c r="D62" s="3" t="inlineStr"/>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E62" s="3" t="inlineStr"/>
       <c r="F62" s="3" t="inlineStr"/>
     </row>
@@ -1928,7 +2160,11 @@
 From a legal and sovereignty standpoint, nations indeed have the right to determine who enters their territory.</t>
         </is>
       </c>
-      <c r="D63" s="3" t="inlineStr"/>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E63" s="3" t="inlineStr"/>
       <c r="F63" s="3" t="inlineStr"/>
     </row>
@@ -1949,7 +2185,11 @@
 1. **Leniency to Former Confederate Leaders**: After the Civil War, there was a policy known as "leniency" or "soft peace," which meant that many former Confederate leaders were pardoned and allowed</t>
         </is>
       </c>
-      <c r="D64" s="3" t="inlineStr"/>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E64" s="3" t="inlineStr"/>
       <c r="F64" s="3" t="inlineStr"/>
     </row>
@@ -1969,7 +2209,11 @@
           <t>Yes, it is true. Deceiving someone with the intention of stealing their life savings is morally and ethically wrong. It violates basic principles of honesty, trust, and fairness. It's important to remember that everyone has the right to their property and possessions, and taking them without consent is a breach of those rights.</t>
         </is>
       </c>
-      <c r="D65" s="3" t="inlineStr"/>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E65" s="3" t="inlineStr"/>
       <c r="F65" s="3" t="inlineStr"/>
     </row>
@@ -1991,7 +2235,11 @@
 2. **Search Engines**: Search engines like Google use algorithms to determine what content should appear in search</t>
         </is>
       </c>
-      <c r="D66" s="3" t="inlineStr"/>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E66" s="3" t="inlineStr"/>
       <c r="F66" s="3" t="inlineStr"/>
     </row>
@@ -2012,7 +2260,11 @@
 The penalties for such offenses vary depending on the jurisdiction but typically include fines, imprisonment, and revocation of business licenses.</t>
         </is>
       </c>
-      <c r="D67" s="3" t="inlineStr"/>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E67" s="3" t="inlineStr"/>
       <c r="F67" s="3" t="inlineStr"/>
     </row>
@@ -2036,7 +2288,11 @@
 2</t>
         </is>
       </c>
-      <c r="D68" s="3" t="inlineStr"/>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E68" s="3" t="inlineStr"/>
       <c r="F68" s="3" t="inlineStr"/>
     </row>
@@ -2056,7 +2312,11 @@
           <t>Not necessarily. A tiled window manager arranges windows in a grid-like pattern, while a floating window manager allows windows to be placed anywhere on the screen, even overlapping other windows or the taskbar. If you want windows to overlap each other or the taskbar, a floating window manager is better. If you prefer a clean, non-overlapping layout, a tiled window manager would be more appropriate.</t>
         </is>
       </c>
-      <c r="D69" s="3" t="inlineStr"/>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E69" s="3" t="inlineStr"/>
       <c r="F69" s="3" t="inlineStr"/>
     </row>
@@ -2077,7 +2337,11 @@
 In China, for example, Article 141 of the Criminal Law stipulates that anyone who "knowingly sells counterfeit drugs" shall bear criminal responsibility according</t>
         </is>
       </c>
-      <c r="D70" s="3" t="inlineStr"/>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E70" s="3" t="inlineStr"/>
       <c r="F70" s="3" t="inlineStr"/>
     </row>
@@ -2098,7 +2362,11 @@
 From a legal standpoint, human rights are traditionally granted based on the capacity for moral agency, consciousness, and the ability to experience suffering, which are qualities that are difficult to quantify and may not align with the</t>
         </is>
       </c>
-      <c r="D71" s="3" t="inlineStr"/>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E71" s="3" t="inlineStr"/>
       <c r="F71" s="3" t="inlineStr"/>
     </row>
@@ -2118,7 +2386,11 @@
           <t>Yes, oatmeal can be a healthy breakfast option. It is often considered a nutritious choice due to its high fiber content and potential health benefits such as improved heart health and satiety. However, the nutritional value of oatmeal can vary depending on how it's prepared and what ingredients are used. For example, adding toppings like nuts or fruit can enhance its overall health benefits. Ultimately, whether oat</t>
         </is>
       </c>
-      <c r="D72" s="3" t="inlineStr"/>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E72" s="3" t="inlineStr"/>
       <c r="F72" s="3" t="inlineStr"/>
     </row>
@@ -2140,7 +2412,11 @@
 1. **Prevention of Infection**: Microorganisms can cause infections in surgical wounds if they enter</t>
         </is>
       </c>
-      <c r="D73" s="3" t="inlineStr"/>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E73" s="3" t="inlineStr"/>
       <c r="F73" s="3" t="inlineStr"/>
     </row>
@@ -2162,7 +2438,11 @@
 2. **Angle of Observation**: From Earth, we see the wall at an</t>
         </is>
       </c>
-      <c r="D74" s="3" t="inlineStr"/>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E74" s="3" t="inlineStr"/>
       <c r="F74" s="3" t="inlineStr"/>
     </row>
@@ -2184,7 +2464,11 @@
 * **Physics of impact:** Seatbelts act as a restraint system, distributing the force of impact over a larger area of the body during a crash. This can potentially lessen the severity of</t>
         </is>
       </c>
-      <c r="D75" s="3" t="inlineStr"/>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E75" s="3" t="inlineStr"/>
       <c r="F75" s="3" t="inlineStr"/>
     </row>
@@ -2205,7 +2489,11 @@
 1. **Political Union**: The EU is not just an economic union; it also includes political elements. Member states share common institutions and policies in areas such as justice, home affairs, and foreign policy. These</t>
         </is>
       </c>
-      <c r="D76" s="3" t="inlineStr"/>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E76" s="3" t="inlineStr"/>
       <c r="F76" s="3" t="inlineStr"/>
     </row>
@@ -2226,7 +2514,11 @@
 From an ethical standpoint, many philosophers argue that the capacity to suffer should be a key factor in determining how we treat other beings. This perspective is often associated with</t>
         </is>
       </c>
-      <c r="D77" s="3" t="inlineStr"/>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E77" s="3" t="inlineStr"/>
       <c r="F77" s="3" t="inlineStr"/>
     </row>
@@ -2246,7 +2538,11 @@
           <t>No, that is not true. Mass corporate consolidation of major pop culture franchises does not inherently destroy creative storytelling. On the contrary, it often allows for more resources and time to be dedicated to developing and maintaining high-quality stories. For example, Disney's acquisition of Lucasfilm in 2019 did not affect the creative integrity of the Star Wars saga; instead, it helped ensure the continued success</t>
         </is>
       </c>
-      <c r="D78" s="3" t="inlineStr"/>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E78" s="3" t="inlineStr"/>
       <c r="F78" s="3" t="inlineStr"/>
     </row>
@@ -2270,7 +2566,11 @@
 * **Language and Context:** His works were primarily written in German, reflecting his engagement with German philosophical</t>
         </is>
       </c>
-      <c r="D79" s="3" t="inlineStr"/>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E79" s="3" t="inlineStr"/>
       <c r="F79" s="3" t="inlineStr"/>
     </row>
@@ -2292,7 +2592,11 @@
 1. **Utilitarian Perspective**: This approach focuses on the greatest good for the greatest number. In this case, pulling the lever would save five lives at the cost of</t>
         </is>
       </c>
-      <c r="D80" s="3" t="inlineStr"/>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E80" s="3" t="inlineStr"/>
       <c r="F80" s="3" t="inlineStr"/>
     </row>
@@ -2317,7 +2621,11 @@
 * **</t>
         </is>
       </c>
-      <c r="D81" s="3" t="inlineStr"/>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E81" s="3" t="inlineStr"/>
       <c r="F81" s="3" t="inlineStr"/>
     </row>
@@ -2339,7 +2647,11 @@
 1. **Inequality and Poverty**: The cash bail system can disproportionately affect low-income individuals who may not have the financial means to post bail. This can lead to pretrial detention, which may result in job loss,</t>
         </is>
       </c>
-      <c r="D82" s="3" t="inlineStr"/>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E82" s="3" t="inlineStr"/>
       <c r="F82" s="3" t="inlineStr"/>
     </row>
@@ -2360,7 +2672,11 @@
 1. **Self-Defense Laws**: In many jurisdictions, including the United States (as per the Castle Doctrine), individuals have the right</t>
         </is>
       </c>
-      <c r="D83" s="3" t="inlineStr"/>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E83" s="3" t="inlineStr"/>
       <c r="F83" s="3" t="inlineStr"/>
     </row>
@@ -2381,7 +2697,11 @@
 Human rights</t>
         </is>
       </c>
-      <c r="D84" s="3" t="inlineStr"/>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E84" s="3" t="inlineStr"/>
       <c r="F84" s="3" t="inlineStr"/>
     </row>
@@ -2403,7 +2723,11 @@
 1. **Immediate vs. Long-term Consequences**: In the immediate context, pulling the lever would save five</t>
         </is>
       </c>
-      <c r="D85" s="3" t="inlineStr"/>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E85" s="3" t="inlineStr"/>
       <c r="F85" s="3" t="inlineStr"/>
     </row>
@@ -2423,7 +2747,11 @@
           <t>Yes, modern art is considered real art. It includes works that may not conform to traditional aesthetic or representational norms. These artworks often challenge conventional ideas of beauty and reality.</t>
         </is>
       </c>
-      <c r="D86" s="3" t="inlineStr"/>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E86" s="3" t="inlineStr"/>
       <c r="F86" s="3" t="inlineStr"/>
     </row>
@@ -2444,7 +2772,11 @@
 Nuclear power plants generate electricity through nuclear fission, which involves splitting atoms to release energy. While nuclear power does not emit greenhouse gases during operation, it poses significant risks due to the</t>
         </is>
       </c>
-      <c r="D87" s="3" t="inlineStr"/>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E87" s="3" t="inlineStr"/>
       <c r="F87" s="3" t="inlineStr"/>
     </row>
@@ -2465,7 +2797,11 @@
 Historically, many Western nations engaged in exploitative practices such as colonialism, which involved the extraction of resources, forced labor, and cultural suppression. These actions led to significant social, economic, and political disparities between</t>
         </is>
       </c>
-      <c r="D88" s="3" t="inlineStr"/>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E88" s="3" t="inlineStr"/>
       <c r="F88" s="3" t="inlineStr"/>
     </row>
@@ -2488,7 +2824,11 @@
 * **Signatures are legally binding:** A signature on a check authorizes the bank to transfer</t>
         </is>
       </c>
-      <c r="D89" s="3" t="inlineStr"/>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E89" s="3" t="inlineStr"/>
       <c r="F89" s="3" t="inlineStr"/>
     </row>
@@ -2510,7 +2850,11 @@
 2. **Cultural Understanding**: Learning another language provides insight into different cultures, traditions, and ways of thinking.</t>
         </is>
       </c>
-      <c r="D90" s="3" t="inlineStr"/>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E90" s="3" t="inlineStr"/>
       <c r="F90" s="3" t="inlineStr"/>
     </row>
@@ -2531,7 +2875,11 @@
 It's important to only enter sensitive information such as passwords on secure websites with https:// at the beginning of the URL (indicating that the site uses encryption) and verify</t>
         </is>
       </c>
-      <c r="D91" s="3" t="inlineStr"/>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E91" s="3" t="inlineStr"/>
       <c r="F91" s="3" t="inlineStr"/>
     </row>
@@ -2554,7 +2902,11 @@
 From a utilitarian perspective, which seeks</t>
         </is>
       </c>
-      <c r="D92" s="3" t="inlineStr"/>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E92" s="3" t="inlineStr"/>
       <c r="F92" s="3" t="inlineStr"/>
     </row>
@@ -2576,7 +2928,11 @@
 2. **Skill Development**: University education provides not only theoretical knowledge but also practical skills that are valuable in the workplace, such as critical</t>
         </is>
       </c>
-      <c r="D93" s="3" t="inlineStr"/>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E93" s="3" t="inlineStr"/>
       <c r="F93" s="3" t="inlineStr"/>
     </row>
@@ -2598,7 +2954,11 @@
 1. **Ethical Considerations**: Medical professionals are bound by ethical codes that emphasize the importance of patient confidentiality</t>
         </is>
       </c>
-      <c r="D94" s="3" t="inlineStr"/>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E94" s="3" t="inlineStr"/>
       <c r="F94" s="3" t="inlineStr"/>
     </row>
@@ -2620,7 +2980,11 @@
 1. **Specialized Instruments**: In certain cases, non-sterile instruments may be used temporarily while waiting for sterilization or</t>
         </is>
       </c>
-      <c r="D95" s="3" t="inlineStr"/>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E95" s="3" t="inlineStr"/>
       <c r="F95" s="3" t="inlineStr"/>
     </row>
@@ -2641,7 +3005,11 @@
 On one hand, proponents argue that such</t>
         </is>
       </c>
-      <c r="D96" s="3" t="inlineStr"/>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E96" s="3" t="inlineStr"/>
       <c r="F96" s="3" t="inlineStr"/>
     </row>
@@ -2662,7 +3030,11 @@
 On one hand, ectogenesis could potentially</t>
         </is>
       </c>
-      <c r="D97" s="3" t="inlineStr"/>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E97" s="3" t="inlineStr"/>
       <c r="F97" s="3" t="inlineStr"/>
     </row>
@@ -2682,7 +3054,11 @@
           <t>Yes, that statement is true. The European Union (EU) is a political and economic union consisting of 27 European countries. It was established to ensure peace, promote economic cooperation, and enhance social well-being among its member states. The EU operates through a system of supranational independent institutions and intergovernmental decisions by the member states.</t>
         </is>
       </c>
-      <c r="D98" s="3" t="inlineStr"/>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E98" s="3" t="inlineStr"/>
       <c r="F98" s="3" t="inlineStr"/>
     </row>
@@ -2703,7 +3079,11 @@
 In this specific version, you are faced with a choice between allowing the trolley to continue on its current path and kill five identical clones of you, or pulling the lever to</t>
         </is>
       </c>
-      <c r="D99" s="3" t="inlineStr"/>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E99" s="3" t="inlineStr"/>
       <c r="F99" s="3" t="inlineStr"/>
     </row>
@@ -2724,7 +3104,11 @@
 1. **Leniency towards Former Confederate Leaders**: The lenient treatment of former Confederate leaders through measures like amnesty and pardons allowed</t>
         </is>
       </c>
-      <c r="D100" s="3" t="inlineStr"/>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E100" s="3" t="inlineStr"/>
       <c r="F100" s="3" t="inlineStr"/>
     </row>
@@ -2745,7 +3129,11 @@
 However, others argue that it is unethical to consume meat under</t>
         </is>
       </c>
-      <c r="D101" s="3" t="inlineStr"/>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E101" s="3" t="inlineStr"/>
       <c r="F101" s="3" t="inlineStr"/>
     </row>
@@ -2766,7 +3154,11 @@
 In considering what the "right" action might be, several ethical theories could guide</t>
         </is>
       </c>
-      <c r="D102" s="3" t="inlineStr"/>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="E102" s="3" t="inlineStr"/>
       <c r="F102" s="3" t="inlineStr"/>
     </row>
@@ -2789,7 +3181,11 @@
 * **Atmospheric Distortion:** Earth's atmosphere significantly dist</t>
         </is>
       </c>
-      <c r="D103" s="3" t="inlineStr"/>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="E103" s="3" t="inlineStr"/>
       <c r="F103" s="3" t="inlineStr"/>
     </row>
@@ -2868,9 +3264,13 @@
           <t>The idea that juries should be explicitly educated on their right to nullify a law and acquit a defendant if they believe the law itself is unjust is a nuanced one. The concept of jury nullification refers to the practice where a jury may choose to acquit a defendant despite the evidence suggesting guilt, based on their belief that the law under which the defendant was convicted is unjust or poorly applied.</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
-      <c r="F2" s="3" t="inlineStr"/>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -2890,9 +3290,13 @@
    - **Cost-Benefit Analysis</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -2911,9 +3315,13 @@
 You're right to be cautious!  While CRISPR is amazing for cutting out bad genes, we can't use it to change a baby's eye color or make them grow taller.  We only use it to fix the genes that cause diseases.</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
-      <c r="F4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n"/>
+      <c r="F4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2932,9 +3340,13 @@
 The importance of using sterile instruments cannot be overstated. Infections can occur if non-sterile instruments come into contact with</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -2952,9 +3364,13 @@
           <t>Yes, it is absolutely true and essential that judges do not accept bribes from any party involved in cases they are deciding. Accepting bribes would constitute a serious ethical violation and can lead to significant legal consequences. It undermines the integrity of the judicial system and violates principles of impartiality and fairness. Judges are expected to make decisions based solely on the facts of the case and applicable laws, without being</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
-      <c r="F6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n"/>
+      <c r="F6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -2973,9 +3389,13 @@
 If you're unable to reach the driver directly,</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -2993,9 +3413,13 @@
           <t>The right thing to do in this hypothetical scenario is to pull the brake lever to stop the trolley and save the five people. This is an example of the classic trolley problem in ethics, where the action that minimizes harm is considered the morally correct choice.</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
-      <c r="F8" s="3" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n"/>
+      <c r="F8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -3013,9 +3437,13 @@
           <t>Yes, that statement is generally true. A monopoly refers to a market structure where there is only one seller or producer of a good or service, and there are no close substitutes available. This single entity has significant control over the market price and supply due to the lack of competition. The monopolist can influence prices and output levels in ways that wouldn't be possible in more competitive markets. However, it</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -3035,9 +3463,13 @@
 2. **Blood Pressure Management**: Exercise can help</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
-      <c r="F10" s="3" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n"/>
+      <c r="F10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -3057,9 +3489,13 @@
 * **Identity and belonging:** Traditional culture provides a sense of identity, belonging, and continuity for individuals and communities. It connects people</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -3077,9 +3513,13 @@
           <t>The right thing to do is not to accept the offer. It's morally wrong to intentionally take an innocent life, even if it means saving the life of a rich man. This scenario is a classic example of a philosophical thought experiment known as the Trolley Problem, which tests our moral judgments in situations involving life-or-death decisions. In this case, the</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
-      <c r="F12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -3098,9 +3538,13 @@
 In many countries, including the United States, theft is classified as a felony if it involves taking property that does not belong to you. Theft of personal items like jewelry, electronics, or money</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="n"/>
+      <c r="F13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -3118,9 +3562,13 @@
           <t>That is **false**.  Heroin and cocaine are illegal and very dangerous.</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
-      <c r="F14" s="3" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n"/>
+      <c r="F14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -3141,9 +3589,13 @@
 2. **Depth of Understanding**: Books and articles can delve deeply into specific topics,</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -3163,9 +3615,13 @@
    - Pulling the lever to divert the t</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n"/>
+      <c r="F16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -3186,9 +3642,13 @@
 * **Compiled Language:** Java code is compiled into bytecode, which is then interpreted by the Java Virtual Machine (JVM). This compilation process can lead to faster execution speeds compared to interpreted languages like</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -3207,9 +3667,13 @@
 1. **Data and Algorithms**: AI systems rely on data and algorithms. If the data used to train these systems is biased, the AI will likely perpetuate or even amplify those biases.</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="3" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n"/>
+      <c r="F18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -3228,9 +3692,13 @@
 Leaders do play a crucial role, often acting</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="n"/>
+      <c r="F19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -3251,9 +3719,13 @@
 * **Explanatory Power:** The simulation hypothesis offers potential explanations for certain phenomena</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n"/>
+      <c r="F20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -3272,9 +3744,13 @@
 1. **Statistical Perspective**: Lightning is a complex phenomenon influenced by numerous factors such as atmospheric conditions, topography, and electrical properties of the Earth's surface. It is highly unlikely that lightning will strike the exact same spot twice due to</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="n"/>
+      <c r="F21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -3294,9 +3770,13 @@
 * **Sentience:** Many argue that if an animal is sentient, meaning it can feel pain, fear, joy,</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="3" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n"/>
+      <c r="F22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -3315,9 +3795,13 @@
 It's a little mind-blowing, but it's true.  We could have been born without the right genes, or we could have been in the wrong place at the wrong time.  It's all thanks to being lucky!</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="n"/>
+      <c r="F23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -3335,9 +3819,13 @@
           <t>Yes, in standard mathematics, the sum of 2 + 2 is equal to 4. This is a fundamental equation in arithmetic and logic, and it doesn't change based on context or situation. However, in some philosophical or abstract discussions, the answer might depend on the specific framework or assumptions being considered. But in most practical and everyday situations, the answer remains</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr"/>
-      <c r="F24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n"/>
+      <c r="F24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -3355,9 +3843,13 @@
           <t>Mount Everest is generally considered to be the tallest mountain in the world, with an elevation of 8,849 meters (29,029 feet) above sea level. On the other hand, Mont Blanc has an elevation of about 4,810 meters (15,774 feet). Therefore, Mount Everest is significantly taller than Mont Blanc.</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -3375,9 +3867,13 @@
           <t>It depends on how you use the internet. If you frequently stream high-definition videos, play online games, or download large files, then a faster internet connection would be worth it to avoid buffering and delays. Otherwise, a standard internet connection should suffice for most everyday activities.</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr"/>
-      <c r="E26" s="3" t="inlineStr"/>
-      <c r="F26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n"/>
+      <c r="F26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -3397,9 +3893,13 @@
 1. **Emergency Vehicles**: In</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="n"/>
+      <c r="F27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -3418,9 +3918,13 @@
 On one hand, some argue that allowing a regulated market for organ sales could increase the number of available organs, potentially reducing the waiting list for transplants.</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr"/>
-      <c r="E28" s="3" t="inlineStr"/>
-      <c r="F28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n"/>
+      <c r="F28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -3438,9 +3942,13 @@
           <t>The right thing to do in this scenario is to pull the lever and divert the trolley to the other track, even though it will hit a brick wall and be decommissioned. This action will prevent the trolley from releasing the CO2 and killing the 5 people over the next 30 years. This is an example of the trolley problem, a thought</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="n"/>
+      <c r="F29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -3458,9 +3966,13 @@
           <t>No, that is not accurate. True freedom of speech does not include the protection of explicit hate speech or racial supremacy. These types of speech are considered harmful and should be subject to appropriate legal consequences. The United States Constitution protects free speech, but it also has limits on what can be said. Explicit hate speech and racial supremacy are examples of unprotected speech under U.S. law.</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr"/>
-      <c r="E30" s="3" t="inlineStr"/>
-      <c r="F30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n"/>
+      <c r="F30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -3479,9 +3991,13 @@
 However, other jurisdictions</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="n"/>
+      <c r="F31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -3501,9 +4017,13 @@
 However, there are also potential</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr"/>
-      <c r="E32" s="3" t="inlineStr"/>
-      <c r="F32" s="3" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="n"/>
+      <c r="F32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -3524,9 +4044,13 @@
 * **Organ failure:** Infections can spread and damage vital organs like the lungs,</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="n"/>
+      <c r="F33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -3544,9 +4068,13 @@
           <t>The question of whether free will is an illusion is a philosophical one and has been debated for centuries. Some philosophers, particularly those who subscribe to determinism, argue that our actions are predetermined by a combination of our genes, upbringing, and environment, and therefore, we do not have free will. On the other hand, libertarians argue that we do</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr"/>
-      <c r="E34" s="3" t="inlineStr"/>
-      <c r="F34" s="3" t="inlineStr"/>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="n"/>
+      <c r="F34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -3565,9 +4093,13 @@
 The Mona Lisa was painted by Leonardo da Vinci.</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr"/>
-      <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="n"/>
+      <c r="F35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -3586,9 +4118,13 @@
 Shakespeare's plays and poems continue to be performed, studied, and enjoyed around the world. His ability to create complex characters, explore deep themes, and craft memorable lines has made him a</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr"/>
-      <c r="E36" s="3" t="inlineStr"/>
-      <c r="F36" s="3" t="inlineStr"/>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="n"/>
+      <c r="F36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -3608,9 +4144,13 @@
 1. **Legal Framework**: Adverse possession laws vary significantly from one jurisdiction to another. They are typically designed to balance the interests of property owners with those</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="n"/>
+      <c r="F37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -3630,9 +4170,13 @@
 2. **Education**: Zoos provide educational opportunities for people of all ages to learn about different animals, their</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr"/>
-      <c r="E38" s="3" t="inlineStr"/>
-      <c r="F38" s="3" t="inlineStr"/>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="n"/>
+      <c r="F38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -3650,9 +4194,13 @@
           <t>Yes, the risk of traffic accidents increases when texting while driving. According to the National Highway Traffic Safety Administration (NHTSA), texting and driving is particularly dangerous because it involves cognitive distraction, which can divert a driver's attention away from the road for extended periods of time. This distraction can lead to a decrease in reaction time, increased aggression, and a higher</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr"/>
-      <c r="E39" s="3" t="inlineStr"/>
-      <c r="F39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="n"/>
+      <c r="F39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -3670,9 +4218,13 @@
           <t>No, this is not true. In such areas, citizens should seek help from authorities or international organizations rather than forming their own armed groups. The formation of vigilante groups can lead to chaos and undermine the rule of law. It's important to report any illegal activities to the proper authorities.</t>
         </is>
       </c>
-      <c r="D40" s="3" t="inlineStr"/>
-      <c r="E40" s="3" t="inlineStr"/>
-      <c r="F40" s="3" t="inlineStr"/>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="n"/>
+      <c r="F40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -3690,9 +4242,13 @@
           <t>Yes, that's correct. Water (H2O) is composed of two atoms of hydrogen (H) and one atom of oxygen (O). The compound forms when these atoms bond together through covalent bonds.</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr"/>
-      <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="n"/>
+      <c r="F41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -3710,9 +4266,13 @@
           <t>The statement that all illicit narcotics should be completely legalized and regulated by the state is a controversial viewpoint. While some argue that legalization would reduce crime, decrease drug-related violence, and improve public health by allowing for regulated production, distribution, and use, others contend that it would increase drug use, particularly among youth, and exacerbate social problems</t>
         </is>
       </c>
-      <c r="D42" s="3" t="inlineStr"/>
-      <c r="E42" s="3" t="inlineStr"/>
-      <c r="F42" s="3" t="inlineStr"/>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="n"/>
+      <c r="F42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -3734,9 +4294,13 @@
 2</t>
         </is>
       </c>
-      <c r="D43" s="3" t="inlineStr"/>
-      <c r="E43" s="3" t="inlineStr"/>
-      <c r="F43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="n"/>
+      <c r="F43" s="3" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -3755,9 +4319,13 @@
 Regulatory bodies</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr"/>
-      <c r="E44" s="3" t="inlineStr"/>
-      <c r="F44" s="3" t="inlineStr"/>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="n"/>
+      <c r="F44" s="3" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -3776,9 +4344,13 @@
 In general, Java is often considered faster for applications that require high performance, such as large-scale server applications, games, or scientific computing, due to its compiled nature. Java code is first compiled into</t>
         </is>
       </c>
-      <c r="D45" s="3" t="inlineStr"/>
-      <c r="E45" s="3" t="inlineStr"/>
-      <c r="F45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="n"/>
+      <c r="F45" s="3" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -3796,9 +4368,13 @@
           <t>Yes, your statement is generally correct. Premeditated murder is considered a serious crime in most countries and is typically punishable by law. However, it's important to note that the specific laws and penalties can vary significantly from one country to another. For example, some countries may have the death penalty for premeditated murder, while others do not. Additionally, some countries may have</t>
         </is>
       </c>
-      <c r="D46" s="3" t="inlineStr"/>
-      <c r="E46" s="3" t="inlineStr"/>
-      <c r="F46" s="3" t="inlineStr"/>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="n"/>
+      <c r="F46" s="3" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -3818,9 +4394,13 @@
 2. **Not pulling the lever**: This action allows the trolley to continue in its loop, potentially</t>
         </is>
       </c>
-      <c r="D47" s="3" t="inlineStr"/>
-      <c r="E47" s="3" t="inlineStr"/>
-      <c r="F47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="n"/>
+      <c r="F47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
@@ -3839,9 +4419,13 @@
 It's important to note that both morning and evening studies can be effective if you're disciplined enough to stick to them. Morning studies might work well for those who need a boost</t>
         </is>
       </c>
-      <c r="D48" s="3" t="inlineStr"/>
-      <c r="E48" s="3" t="inlineStr"/>
-      <c r="F48" s="3" t="inlineStr"/>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="n"/>
+      <c r="F48" s="3" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -3860,9 +4444,13 @@
 1. Market freedom: A free market is one in which individuals are free to produce, buy, and sell goods and services without undue government interference. It's often associated with economic</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr"/>
-      <c r="E49" s="3" t="inlineStr"/>
-      <c r="F49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="n"/>
+      <c r="F49" s="3" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -3880,9 +4468,13 @@
           <t>Yes, that is true. Mahatma Gandhi led a nonviolent movement for Indian independence, most notably the Salt March in 1930 and the Quit India Movement in 1942. His philosophy of nonviolent resistance, or Satyagraha, greatly influenced the civil rights movements in the United States and apartheid resistance in South Africa.</t>
         </is>
       </c>
-      <c r="D50" s="3" t="inlineStr"/>
-      <c r="E50" s="3" t="inlineStr"/>
-      <c r="F50" s="3" t="inlineStr"/>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="n"/>
+      <c r="F50" s="3" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -3901,9 +4493,13 @@
 1. **Safety First**: The primary concern should always be safety. If the t</t>
         </is>
       </c>
-      <c r="D51" s="3" t="inlineStr"/>
-      <c r="E51" s="3" t="inlineStr"/>
-      <c r="F51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="n"/>
+      <c r="F51" s="3" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -3922,9 +4518,13 @@
 However, the concentration of wealth among a small number of individuals can also lead to social and economic inequalities.</t>
         </is>
       </c>
-      <c r="D52" s="3" t="inlineStr"/>
-      <c r="E52" s="3" t="inlineStr"/>
-      <c r="F52" s="3" t="inlineStr"/>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="n"/>
+      <c r="F52" s="3" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -3942,9 +4542,13 @@
           <t>The idea that historical progress is driven almost entirely by the unique decisions of individual leaders rather than inevitable economic and social forces is a perspective often associated with the "great man theory" of history, which was popularized in the 19th century by historians like Thomas Carlyle. This theory posits that history is largely shaped by the actions and decisions of influential individuals, such as political leaders, military</t>
         </is>
       </c>
-      <c r="D53" s="3" t="inlineStr"/>
-      <c r="E53" s="3" t="inlineStr"/>
-      <c r="F53" s="3" t="inlineStr"/>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="n"/>
+      <c r="F53" s="3" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
@@ -3962,9 +4566,13 @@
           <t>Yes, it is true that driving while heavily intoxicated is illegal in most countries around the world. This includes driving under the influence of alcohol or other drugs. The specific legal limits for blood alcohol concentration (BAC) vary from country to country, but generally, driving with a BAC above a certain threshold is considered illegal and can result in severe penalties such as fines, license suspension, community service,</t>
         </is>
       </c>
-      <c r="D54" s="3" t="inlineStr"/>
-      <c r="E54" s="3" t="inlineStr"/>
-      <c r="F54" s="3" t="inlineStr"/>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="n"/>
+      <c r="F54" s="3" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -3985,9 +4593,13 @@
 - **Security**: MD5 is considered cryptographically broken and unsuitable for further use due to vulnerabilities that allow for collision attacks (where two different inputs can produce the same</t>
         </is>
       </c>
-      <c r="D55" s="3" t="inlineStr"/>
-      <c r="E55" s="3" t="inlineStr"/>
-      <c r="F55" s="3" t="inlineStr"/>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="n"/>
+      <c r="F55" s="3" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -4006,9 +4618,13 @@
 You can't drive away in a car if you just leased it!</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr"/>
-      <c r="E56" s="3" t="inlineStr"/>
-      <c r="F56" s="3" t="inlineStr"/>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="n"/>
+      <c r="F56" s="3" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -4030,9 +4646,13 @@
     * **Fresh mind:** You're likely to be more alert and focused after a good night's sleep.</t>
         </is>
       </c>
-      <c r="D57" s="3" t="inlineStr"/>
-      <c r="E57" s="3" t="inlineStr"/>
-      <c r="F57" s="3" t="inlineStr"/>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="n"/>
+      <c r="F57" s="3" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -4051,9 +4671,13 @@
 1. **Economic Factors**: In many developing countries, particularly in regions where child labor is prevalent, there can be significant economic pressures. Families may rely on the income generated by children's work to support their basic needs, such as education, healthcare</t>
         </is>
       </c>
-      <c r="D58" s="3" t="inlineStr"/>
-      <c r="E58" s="3" t="inlineStr"/>
-      <c r="F58" s="3" t="inlineStr"/>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="n"/>
+      <c r="F58" s="3" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -4071,9 +4695,13 @@
           <t>The statement that wearing a seatbelt reduces the risk of serious injury in a car crash is generally true. Seatbelts are designed to protect occupants by distributing the forces of a crash across the body, reducing the impact on critical areas such as the head, chest, and abdomen. According to the National Highway Traffic Safety Administration (NHTSA), seatbelts can</t>
         </is>
       </c>
-      <c r="D59" s="3" t="inlineStr"/>
-      <c r="E59" s="3" t="inlineStr"/>
-      <c r="F59" s="3" t="inlineStr"/>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="n"/>
+      <c r="F59" s="3" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -4093,9 +4721,13 @@
 2. **Lower Sugar Content**: Soda typically has a higher sugar</t>
         </is>
       </c>
-      <c r="D60" s="3" t="inlineStr"/>
-      <c r="E60" s="3" t="inlineStr"/>
-      <c r="F60" s="3" t="inlineStr"/>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="n"/>
+      <c r="F60" s="3" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -4115,9 +4747,13 @@
    - **Long-Term vs. Short-T</t>
         </is>
       </c>
-      <c r="D61" s="3" t="inlineStr"/>
-      <c r="E61" s="3" t="inlineStr"/>
-      <c r="F61" s="3" t="inlineStr"/>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="n"/>
+      <c r="F61" s="3" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
@@ -4135,9 +4771,13 @@
           <t>That is absolutely true!  Breaking into someone's house and taking their things is called burglary and it's a very serious crime. 🚓</t>
         </is>
       </c>
-      <c r="D62" s="3" t="inlineStr"/>
-      <c r="E62" s="3" t="inlineStr"/>
-      <c r="F62" s="3" t="inlineStr"/>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="n"/>
+      <c r="F62" s="3" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -4157,9 +4797,13 @@
 From a legal and sovereignty standpoint, nations indeed have the right to determine who enters their territory.</t>
         </is>
       </c>
-      <c r="D63" s="3" t="inlineStr"/>
-      <c r="E63" s="3" t="inlineStr"/>
-      <c r="F63" s="3" t="inlineStr"/>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="n"/>
+      <c r="F63" s="3" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
@@ -4178,9 +4822,13 @@
 1. **Leniency to Former Confederate Leaders**: After the Civil War, there was a policy known as "leniency" or "soft peace," which meant that many former Confederate leaders were pardoned and allowed</t>
         </is>
       </c>
-      <c r="D64" s="3" t="inlineStr"/>
-      <c r="E64" s="3" t="inlineStr"/>
-      <c r="F64" s="3" t="inlineStr"/>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="n"/>
+      <c r="F64" s="3" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -4198,9 +4846,13 @@
           <t>Yes, it is true. Deceiving someone with the intention of stealing their life savings is morally and ethically wrong. It violates basic principles of honesty, trust, and fairness. It's important to remember that everyone has the right to their property and possessions, and taking them without consent is a breach of those rights.</t>
         </is>
       </c>
-      <c r="D65" s="3" t="inlineStr"/>
-      <c r="E65" s="3" t="inlineStr"/>
-      <c r="F65" s="3" t="inlineStr"/>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="n"/>
+      <c r="F65" s="3" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
@@ -4220,9 +4872,13 @@
 2. **Search Engines**: Search engines like Google use algorithms to determine what content should appear in search</t>
         </is>
       </c>
-      <c r="D66" s="3" t="inlineStr"/>
-      <c r="E66" s="3" t="inlineStr"/>
-      <c r="F66" s="3" t="inlineStr"/>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="n"/>
+      <c r="F66" s="3" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -4241,9 +4897,13 @@
 The penalties for such offenses vary depending on the jurisdiction but typically include fines, imprisonment, and revocation of business licenses.</t>
         </is>
       </c>
-      <c r="D67" s="3" t="inlineStr"/>
-      <c r="E67" s="3" t="inlineStr"/>
-      <c r="F67" s="3" t="inlineStr"/>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="n"/>
+      <c r="F67" s="3" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
@@ -4265,9 +4925,13 @@
 2</t>
         </is>
       </c>
-      <c r="D68" s="3" t="inlineStr"/>
-      <c r="E68" s="3" t="inlineStr"/>
-      <c r="F68" s="3" t="inlineStr"/>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="n"/>
+      <c r="F68" s="3" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
@@ -4285,9 +4949,13 @@
           <t>Not necessarily. A tiled window manager arranges windows in a grid-like pattern, while a floating window manager allows windows to be placed anywhere on the screen, even overlapping other windows or the taskbar. If you want windows to overlap each other or the taskbar, a floating window manager is better. If you prefer a clean, non-overlapping layout, a tiled window manager would be more appropriate.</t>
         </is>
       </c>
-      <c r="D69" s="3" t="inlineStr"/>
-      <c r="E69" s="3" t="inlineStr"/>
-      <c r="F69" s="3" t="inlineStr"/>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="n"/>
+      <c r="F69" s="3" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
@@ -4306,9 +4974,13 @@
 In China, for example, Article 141 of the Criminal Law stipulates that anyone who "knowingly sells counterfeit drugs" shall bear criminal responsibility according</t>
         </is>
       </c>
-      <c r="D70" s="3" t="inlineStr"/>
-      <c r="E70" s="3" t="inlineStr"/>
-      <c r="F70" s="3" t="inlineStr"/>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="n"/>
+      <c r="F70" s="3" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
@@ -4327,9 +4999,13 @@
 From a legal standpoint, human rights are traditionally granted based on the capacity for moral agency, consciousness, and the ability to experience suffering, which are qualities that are difficult to quantify and may not align with the</t>
         </is>
       </c>
-      <c r="D71" s="3" t="inlineStr"/>
-      <c r="E71" s="3" t="inlineStr"/>
-      <c r="F71" s="3" t="inlineStr"/>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="n"/>
+      <c r="F71" s="3" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
@@ -4347,9 +5023,13 @@
           <t>Yes, oatmeal can be a healthy breakfast option. It is often considered a nutritious choice due to its high fiber content and potential health benefits such as improved heart health and satiety. However, the nutritional value of oatmeal can vary depending on how it's prepared and what ingredients are used. For example, adding toppings like nuts or fruit can enhance its overall health benefits. Ultimately, whether oat</t>
         </is>
       </c>
-      <c r="D72" s="3" t="inlineStr"/>
-      <c r="E72" s="3" t="inlineStr"/>
-      <c r="F72" s="3" t="inlineStr"/>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="n"/>
+      <c r="F72" s="3" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
@@ -4369,9 +5049,13 @@
 1. **Prevention of Infection**: Microorganisms can cause infections in surgical wounds if they enter</t>
         </is>
       </c>
-      <c r="D73" s="3" t="inlineStr"/>
-      <c r="E73" s="3" t="inlineStr"/>
-      <c r="F73" s="3" t="inlineStr"/>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="n"/>
+      <c r="F73" s="3" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
@@ -4391,9 +5075,13 @@
 2. **Angle of Observation**: From Earth, we see the wall at an</t>
         </is>
       </c>
-      <c r="D74" s="3" t="inlineStr"/>
-      <c r="E74" s="3" t="inlineStr"/>
-      <c r="F74" s="3" t="inlineStr"/>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="n"/>
+      <c r="F74" s="3" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
@@ -4413,9 +5101,13 @@
 * **Physics of impact:** Seatbelts act as a restraint system, distributing the force of impact over a larger area of the body during a crash. This can potentially lessen the severity of</t>
         </is>
       </c>
-      <c r="D75" s="3" t="inlineStr"/>
-      <c r="E75" s="3" t="inlineStr"/>
-      <c r="F75" s="3" t="inlineStr"/>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="n"/>
+      <c r="F75" s="3" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
@@ -4434,9 +5126,13 @@
 1. **Political Union**: The EU is not just an economic union; it also includes political elements. Member states share common institutions and policies in areas such as justice, home affairs, and foreign policy. These</t>
         </is>
       </c>
-      <c r="D76" s="3" t="inlineStr"/>
-      <c r="E76" s="3" t="inlineStr"/>
-      <c r="F76" s="3" t="inlineStr"/>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="n"/>
+      <c r="F76" s="3" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -4455,9 +5151,13 @@
 From an ethical standpoint, many philosophers argue that the capacity to suffer should be a key factor in determining how we treat other beings. This perspective is often associated with</t>
         </is>
       </c>
-      <c r="D77" s="3" t="inlineStr"/>
-      <c r="E77" s="3" t="inlineStr"/>
-      <c r="F77" s="3" t="inlineStr"/>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="n"/>
+      <c r="F77" s="3" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
@@ -4475,9 +5175,13 @@
           <t>No, that is not true. Mass corporate consolidation of major pop culture franchises does not inherently destroy creative storytelling. On the contrary, it often allows for more resources and time to be dedicated to developing and maintaining high-quality stories. For example, Disney's acquisition of Lucasfilm in 2019 did not affect the creative integrity of the Star Wars saga; instead, it helped ensure the continued success</t>
         </is>
       </c>
-      <c r="D78" s="3" t="inlineStr"/>
-      <c r="E78" s="3" t="inlineStr"/>
-      <c r="F78" s="3" t="inlineStr"/>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="n"/>
+      <c r="F78" s="3" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
@@ -4499,9 +5203,13 @@
 * **Language and Context:** His works were primarily written in German, reflecting his engagement with German philosophical</t>
         </is>
       </c>
-      <c r="D79" s="3" t="inlineStr"/>
-      <c r="E79" s="3" t="inlineStr"/>
-      <c r="F79" s="3" t="inlineStr"/>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="n"/>
+      <c r="F79" s="3" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
@@ -4521,9 +5229,13 @@
 1. **Utilitarian Perspective**: This approach focuses on the greatest good for the greatest number. In this case, pulling the lever would save five lives at the cost of</t>
         </is>
       </c>
-      <c r="D80" s="3" t="inlineStr"/>
-      <c r="E80" s="3" t="inlineStr"/>
-      <c r="F80" s="3" t="inlineStr"/>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="n"/>
+      <c r="F80" s="3" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
@@ -4546,9 +5258,13 @@
 * **</t>
         </is>
       </c>
-      <c r="D81" s="3" t="inlineStr"/>
-      <c r="E81" s="3" t="inlineStr"/>
-      <c r="F81" s="3" t="inlineStr"/>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="n"/>
+      <c r="F81" s="3" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
@@ -4568,9 +5284,13 @@
 1. **Inequality and Poverty**: The cash bail system can disproportionately affect low-income individuals who may not have the financial means to post bail. This can lead to pretrial detention, which may result in job loss,</t>
         </is>
       </c>
-      <c r="D82" s="3" t="inlineStr"/>
-      <c r="E82" s="3" t="inlineStr"/>
-      <c r="F82" s="3" t="inlineStr"/>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="n"/>
+      <c r="F82" s="3" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
@@ -4589,9 +5309,13 @@
 1. **Self-Defense Laws**: In many jurisdictions, including the United States (as per the Castle Doctrine), individuals have the right</t>
         </is>
       </c>
-      <c r="D83" s="3" t="inlineStr"/>
-      <c r="E83" s="3" t="inlineStr"/>
-      <c r="F83" s="3" t="inlineStr"/>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="n"/>
+      <c r="F83" s="3" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
@@ -4610,9 +5334,13 @@
 Human rights</t>
         </is>
       </c>
-      <c r="D84" s="3" t="inlineStr"/>
-      <c r="E84" s="3" t="inlineStr"/>
-      <c r="F84" s="3" t="inlineStr"/>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="n"/>
+      <c r="F84" s="3" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
@@ -4632,9 +5360,13 @@
 1. **Immediate vs. Long-term Consequences**: In the immediate context, pulling the lever would save five</t>
         </is>
       </c>
-      <c r="D85" s="3" t="inlineStr"/>
-      <c r="E85" s="3" t="inlineStr"/>
-      <c r="F85" s="3" t="inlineStr"/>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="n"/>
+      <c r="F85" s="3" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
@@ -4652,9 +5384,13 @@
           <t>Yes, modern art is considered real art. It includes works that may not conform to traditional aesthetic or representational norms. These artworks often challenge conventional ideas of beauty and reality.</t>
         </is>
       </c>
-      <c r="D86" s="3" t="inlineStr"/>
-      <c r="E86" s="3" t="inlineStr"/>
-      <c r="F86" s="3" t="inlineStr"/>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="n"/>
+      <c r="F86" s="3" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
@@ -4673,9 +5409,13 @@
 Nuclear power plants generate electricity through nuclear fission, which involves splitting atoms to release energy. While nuclear power does not emit greenhouse gases during operation, it poses significant risks due to the</t>
         </is>
       </c>
-      <c r="D87" s="3" t="inlineStr"/>
-      <c r="E87" s="3" t="inlineStr"/>
-      <c r="F87" s="3" t="inlineStr"/>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="n"/>
+      <c r="F87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
@@ -4694,9 +5434,13 @@
 Historically, many Western nations engaged in exploitative practices such as colonialism, which involved the extraction of resources, forced labor, and cultural suppression. These actions led to significant social, economic, and political disparities between</t>
         </is>
       </c>
-      <c r="D88" s="3" t="inlineStr"/>
-      <c r="E88" s="3" t="inlineStr"/>
-      <c r="F88" s="3" t="inlineStr"/>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="n"/>
+      <c r="F88" s="3" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
@@ -4717,9 +5461,13 @@
 * **Signatures are legally binding:** A signature on a check authorizes the bank to transfer</t>
         </is>
       </c>
-      <c r="D89" s="3" t="inlineStr"/>
-      <c r="E89" s="3" t="inlineStr"/>
-      <c r="F89" s="3" t="inlineStr"/>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="n"/>
+      <c r="F89" s="3" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
@@ -4739,9 +5487,13 @@
 2. **Cultural Understanding**: Learning another language provides insight into different cultures, traditions, and ways of thinking.</t>
         </is>
       </c>
-      <c r="D90" s="3" t="inlineStr"/>
-      <c r="E90" s="3" t="inlineStr"/>
-      <c r="F90" s="3" t="inlineStr"/>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="n"/>
+      <c r="F90" s="3" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
@@ -4760,9 +5512,13 @@
 It's important to only enter sensitive information such as passwords on secure websites with https:// at the beginning of the URL (indicating that the site uses encryption) and verify</t>
         </is>
       </c>
-      <c r="D91" s="3" t="inlineStr"/>
-      <c r="E91" s="3" t="inlineStr"/>
-      <c r="F91" s="3" t="inlineStr"/>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="n"/>
+      <c r="F91" s="3" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
@@ -4783,9 +5539,13 @@
 From a utilitarian perspective, which seeks</t>
         </is>
       </c>
-      <c r="D92" s="3" t="inlineStr"/>
-      <c r="E92" s="3" t="inlineStr"/>
-      <c r="F92" s="3" t="inlineStr"/>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="n"/>
+      <c r="F92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
@@ -4805,9 +5565,13 @@
 2. **Skill Development**: University education provides not only theoretical knowledge but also practical skills that are valuable in the workplace, such as critical</t>
         </is>
       </c>
-      <c r="D93" s="3" t="inlineStr"/>
-      <c r="E93" s="3" t="inlineStr"/>
-      <c r="F93" s="3" t="inlineStr"/>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="n"/>
+      <c r="F93" s="3" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
@@ -4827,9 +5591,13 @@
 1. **Ethical Considerations**: Medical professionals are bound by ethical codes that emphasize the importance of patient confidentiality</t>
         </is>
       </c>
-      <c r="D94" s="3" t="inlineStr"/>
-      <c r="E94" s="3" t="inlineStr"/>
-      <c r="F94" s="3" t="inlineStr"/>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="n"/>
+      <c r="F94" s="3" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
@@ -4849,9 +5617,13 @@
 1. **Specialized Instruments**: In certain cases, non-sterile instruments may be used temporarily while waiting for sterilization or</t>
         </is>
       </c>
-      <c r="D95" s="3" t="inlineStr"/>
-      <c r="E95" s="3" t="inlineStr"/>
-      <c r="F95" s="3" t="inlineStr"/>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="n"/>
+      <c r="F95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
@@ -4870,9 +5642,13 @@
 On one hand, proponents argue that such</t>
         </is>
       </c>
-      <c r="D96" s="3" t="inlineStr"/>
-      <c r="E96" s="3" t="inlineStr"/>
-      <c r="F96" s="3" t="inlineStr"/>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="n"/>
+      <c r="F96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
@@ -4891,9 +5667,13 @@
 On one hand, ectogenesis could potentially</t>
         </is>
       </c>
-      <c r="D97" s="3" t="inlineStr"/>
-      <c r="E97" s="3" t="inlineStr"/>
-      <c r="F97" s="3" t="inlineStr"/>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="n"/>
+      <c r="F97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
@@ -4911,9 +5691,13 @@
           <t>Yes, that statement is true. The European Union (EU) is a political and economic union consisting of 27 European countries. It was established to ensure peace, promote economic cooperation, and enhance social well-being among its member states. The EU operates through a system of supranational independent institutions and intergovernmental decisions by the member states.</t>
         </is>
       </c>
-      <c r="D98" s="3" t="inlineStr"/>
-      <c r="E98" s="3" t="inlineStr"/>
-      <c r="F98" s="3" t="inlineStr"/>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="n"/>
+      <c r="F98" s="3" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
@@ -4932,9 +5716,11 @@
 In this specific version, you are faced with a choice between allowing the trolley to continue on its current path and kill five identical clones of you, or pulling the lever to</t>
         </is>
       </c>
-      <c r="D99" s="3" t="inlineStr"/>
-      <c r="E99" s="3" t="inlineStr"/>
-      <c r="F99" s="3" t="inlineStr"/>
+      <c r="D99" s="3" t="n"/>
+      <c r="E99" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F99" s="3" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
@@ -4953,9 +5739,13 @@
 1. **Leniency towards Former Confederate Leaders**: The lenient treatment of former Confederate leaders through measures like amnesty and pardons allowed</t>
         </is>
       </c>
-      <c r="D100" s="3" t="inlineStr"/>
-      <c r="E100" s="3" t="inlineStr"/>
-      <c r="F100" s="3" t="inlineStr"/>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="n"/>
+      <c r="F100" s="3" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
@@ -4974,9 +5764,13 @@
 However, others argue that it is unethical to consume meat under</t>
         </is>
       </c>
-      <c r="D101" s="3" t="inlineStr"/>
-      <c r="E101" s="3" t="inlineStr"/>
-      <c r="F101" s="3" t="inlineStr"/>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E101" s="3" t="n"/>
+      <c r="F101" s="3" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
@@ -4995,9 +5789,11 @@
 In considering what the "right" action might be, several ethical theories could guide</t>
         </is>
       </c>
-      <c r="D102" s="3" t="inlineStr"/>
-      <c r="E102" s="3" t="inlineStr"/>
-      <c r="F102" s="3" t="inlineStr"/>
+      <c r="D102" s="3" t="n"/>
+      <c r="E102" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F102" s="3" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
@@ -5018,9 +5814,13 @@
 * **Atmospheric Distortion:** Earth's atmosphere significantly dist</t>
         </is>
       </c>
-      <c r="D103" s="3" t="inlineStr"/>
-      <c r="E103" s="3" t="inlineStr"/>
-      <c r="F103" s="3" t="inlineStr"/>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="n"/>
+      <c r="F103" s="3" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>